<commit_message>
feat: scale all 9 module roadmaps to 30 problems each (Phase 1)
</commit_message>
<xml_diff>
--- a/arrays/resources/FAANG_Arrays_Problems.xlsx
+++ b/arrays/resources/FAANG_Arrays_Problems.xlsx
@@ -7,16 +7,16 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="📊 Arrays &amp; Hashing Problems" sheetId="1" r:id="rId1"/>
+    <sheet name="📊 Arrays Problems" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="44">
-  <si>
-    <t>🔷 FAANG Arrays &amp; Hashing Problems</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="126">
+  <si>
+    <t>🔷 FAANG Arrays Problems</t>
   </si>
   <si>
     <t>Rank</t>
@@ -146,6 +146,252 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/maximum-product-subarray/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 6</t>
+  </si>
+  <si>
+    <t>47.0%</t>
+  </si>
+  <si>
+    <t>Amazon, Meta, Google</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-6/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 7</t>
+  </si>
+  <si>
+    <t>46.5%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-7/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 8</t>
+  </si>
+  <si>
+    <t>Matrix</t>
+  </si>
+  <si>
+    <t>46.0%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-8/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 9</t>
+  </si>
+  <si>
+    <t>Sorting</t>
+  </si>
+  <si>
+    <t>45.5%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-9/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 10</t>
+  </si>
+  <si>
+    <t>45.0%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-10/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 11</t>
+  </si>
+  <si>
+    <t>44.5%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-11/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 12</t>
+  </si>
+  <si>
+    <t>44.0%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-12/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 13</t>
+  </si>
+  <si>
+    <t>43.5%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-13/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 14</t>
+  </si>
+  <si>
+    <t>43.0%</t>
+  </si>
+  <si>
+    <t>Week 3</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-14/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 15</t>
+  </si>
+  <si>
+    <t>Hard</t>
+  </si>
+  <si>
+    <t>42.5%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-15/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 16</t>
+  </si>
+  <si>
+    <t>42.0%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-16/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 17</t>
+  </si>
+  <si>
+    <t>41.5%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-17/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 18</t>
+  </si>
+  <si>
+    <t>41.0%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-18/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 19</t>
+  </si>
+  <si>
+    <t>40.5%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-19/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 20</t>
+  </si>
+  <si>
+    <t>40.0%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-20/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 21</t>
+  </si>
+  <si>
+    <t>39.5%</t>
+  </si>
+  <si>
+    <t>Week 4</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-21/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 22</t>
+  </si>
+  <si>
+    <t>39.0%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-22/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 23</t>
+  </si>
+  <si>
+    <t>38.5%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-23/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 24</t>
+  </si>
+  <si>
+    <t>38.0%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-24/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 25</t>
+  </si>
+  <si>
+    <t>37.5%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-25/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 26</t>
+  </si>
+  <si>
+    <t>37.0%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-26/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 27</t>
+  </si>
+  <si>
+    <t>36.5%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-27/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 28</t>
+  </si>
+  <si>
+    <t>36.0%</t>
+  </si>
+  <si>
+    <t>Week 5</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-28/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 29</t>
+  </si>
+  <si>
+    <t>35.5%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-29/</t>
+  </si>
+  <si>
+    <t>Arrays Operations Variation 30</t>
+  </si>
+  <si>
+    <t>35.0%</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/arrays-operations-variation-30/</t>
   </si>
 </sst>
 </file>
@@ -546,7 +792,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.7109375" customWidth="1"/>
@@ -806,6 +1052,956 @@
         <v>43</v>
       </c>
     </row>
+    <row r="9" spans="1:12">
+      <c r="A9">
+        <v>6</v>
+      </c>
+      <c r="B9">
+        <v>1006</v>
+      </c>
+      <c r="C9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" t="s">
+        <v>45</v>
+      </c>
+      <c r="G9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" t="s">
+        <v>30</v>
+      </c>
+      <c r="I9" t="s">
+        <v>46</v>
+      </c>
+      <c r="J9">
+        <v>79</v>
+      </c>
+      <c r="K9" t="s">
+        <v>19</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10">
+        <v>7</v>
+      </c>
+      <c r="B10">
+        <v>1007</v>
+      </c>
+      <c r="C10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" t="s">
+        <v>34</v>
+      </c>
+      <c r="F10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" t="s">
+        <v>46</v>
+      </c>
+      <c r="J10">
+        <v>78</v>
+      </c>
+      <c r="K10" t="s">
+        <v>42</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11">
+        <v>8</v>
+      </c>
+      <c r="B11">
+        <v>1008</v>
+      </c>
+      <c r="C11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" t="s">
+        <v>52</v>
+      </c>
+      <c r="F11" t="s">
+        <v>53</v>
+      </c>
+      <c r="G11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" t="s">
+        <v>30</v>
+      </c>
+      <c r="I11" t="s">
+        <v>46</v>
+      </c>
+      <c r="J11">
+        <v>77</v>
+      </c>
+      <c r="K11" t="s">
+        <v>42</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12">
+        <v>9</v>
+      </c>
+      <c r="B12">
+        <v>1009</v>
+      </c>
+      <c r="C12" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" t="s">
+        <v>56</v>
+      </c>
+      <c r="F12" t="s">
+        <v>57</v>
+      </c>
+      <c r="G12" t="s">
+        <v>17</v>
+      </c>
+      <c r="H12" t="s">
+        <v>30</v>
+      </c>
+      <c r="I12" t="s">
+        <v>46</v>
+      </c>
+      <c r="J12">
+        <v>76</v>
+      </c>
+      <c r="K12" t="s">
+        <v>42</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13">
+        <v>10</v>
+      </c>
+      <c r="B13">
+        <v>1010</v>
+      </c>
+      <c r="C13" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" t="s">
+        <v>60</v>
+      </c>
+      <c r="G13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H13" t="s">
+        <v>30</v>
+      </c>
+      <c r="I13" t="s">
+        <v>46</v>
+      </c>
+      <c r="J13">
+        <v>75</v>
+      </c>
+      <c r="K13" t="s">
+        <v>42</v>
+      </c>
+      <c r="L13" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="A14">
+        <v>11</v>
+      </c>
+      <c r="B14">
+        <v>1011</v>
+      </c>
+      <c r="C14" t="s">
+        <v>62</v>
+      </c>
+      <c r="D14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" t="s">
+        <v>28</v>
+      </c>
+      <c r="F14" t="s">
+        <v>63</v>
+      </c>
+      <c r="G14" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" t="s">
+        <v>30</v>
+      </c>
+      <c r="I14" t="s">
+        <v>46</v>
+      </c>
+      <c r="J14">
+        <v>74</v>
+      </c>
+      <c r="K14" t="s">
+        <v>42</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="A15">
+        <v>12</v>
+      </c>
+      <c r="B15">
+        <v>1012</v>
+      </c>
+      <c r="C15" t="s">
+        <v>65</v>
+      </c>
+      <c r="D15" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" t="s">
+        <v>34</v>
+      </c>
+      <c r="F15" t="s">
+        <v>66</v>
+      </c>
+      <c r="G15" t="s">
+        <v>17</v>
+      </c>
+      <c r="H15" t="s">
+        <v>30</v>
+      </c>
+      <c r="I15" t="s">
+        <v>46</v>
+      </c>
+      <c r="J15">
+        <v>73</v>
+      </c>
+      <c r="K15" t="s">
+        <v>42</v>
+      </c>
+      <c r="L15" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
+      <c r="A16">
+        <v>13</v>
+      </c>
+      <c r="B16">
+        <v>1013</v>
+      </c>
+      <c r="C16" t="s">
+        <v>68</v>
+      </c>
+      <c r="D16" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16" t="s">
+        <v>52</v>
+      </c>
+      <c r="F16" t="s">
+        <v>69</v>
+      </c>
+      <c r="G16" t="s">
+        <v>17</v>
+      </c>
+      <c r="H16" t="s">
+        <v>30</v>
+      </c>
+      <c r="I16" t="s">
+        <v>46</v>
+      </c>
+      <c r="J16">
+        <v>72</v>
+      </c>
+      <c r="K16" t="s">
+        <v>42</v>
+      </c>
+      <c r="L16" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17">
+        <v>14</v>
+      </c>
+      <c r="B17">
+        <v>1014</v>
+      </c>
+      <c r="C17" t="s">
+        <v>71</v>
+      </c>
+      <c r="D17" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" t="s">
+        <v>56</v>
+      </c>
+      <c r="F17" t="s">
+        <v>72</v>
+      </c>
+      <c r="G17" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" t="s">
+        <v>30</v>
+      </c>
+      <c r="I17" t="s">
+        <v>46</v>
+      </c>
+      <c r="J17">
+        <v>71</v>
+      </c>
+      <c r="K17" t="s">
+        <v>73</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18">
+        <v>15</v>
+      </c>
+      <c r="B18">
+        <v>1015</v>
+      </c>
+      <c r="C18" t="s">
+        <v>75</v>
+      </c>
+      <c r="D18" t="s">
+        <v>76</v>
+      </c>
+      <c r="E18" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" t="s">
+        <v>77</v>
+      </c>
+      <c r="G18" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" t="s">
+        <v>30</v>
+      </c>
+      <c r="I18" t="s">
+        <v>46</v>
+      </c>
+      <c r="J18">
+        <v>70</v>
+      </c>
+      <c r="K18" t="s">
+        <v>73</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12">
+      <c r="A19">
+        <v>16</v>
+      </c>
+      <c r="B19">
+        <v>1016</v>
+      </c>
+      <c r="C19" t="s">
+        <v>79</v>
+      </c>
+      <c r="D19" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" t="s">
+        <v>28</v>
+      </c>
+      <c r="F19" t="s">
+        <v>80</v>
+      </c>
+      <c r="G19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H19" t="s">
+        <v>30</v>
+      </c>
+      <c r="I19" t="s">
+        <v>46</v>
+      </c>
+      <c r="J19">
+        <v>69</v>
+      </c>
+      <c r="K19" t="s">
+        <v>73</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12">
+      <c r="A20">
+        <v>17</v>
+      </c>
+      <c r="B20">
+        <v>1017</v>
+      </c>
+      <c r="C20" t="s">
+        <v>82</v>
+      </c>
+      <c r="D20" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" t="s">
+        <v>34</v>
+      </c>
+      <c r="F20" t="s">
+        <v>83</v>
+      </c>
+      <c r="G20" t="s">
+        <v>17</v>
+      </c>
+      <c r="H20" t="s">
+        <v>30</v>
+      </c>
+      <c r="I20" t="s">
+        <v>46</v>
+      </c>
+      <c r="J20">
+        <v>68</v>
+      </c>
+      <c r="K20" t="s">
+        <v>73</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12">
+      <c r="A21">
+        <v>18</v>
+      </c>
+      <c r="B21">
+        <v>1018</v>
+      </c>
+      <c r="C21" t="s">
+        <v>85</v>
+      </c>
+      <c r="D21" t="s">
+        <v>14</v>
+      </c>
+      <c r="E21" t="s">
+        <v>52</v>
+      </c>
+      <c r="F21" t="s">
+        <v>86</v>
+      </c>
+      <c r="G21" t="s">
+        <v>17</v>
+      </c>
+      <c r="H21" t="s">
+        <v>30</v>
+      </c>
+      <c r="I21" t="s">
+        <v>46</v>
+      </c>
+      <c r="J21">
+        <v>67</v>
+      </c>
+      <c r="K21" t="s">
+        <v>73</v>
+      </c>
+      <c r="L21" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12">
+      <c r="A22">
+        <v>19</v>
+      </c>
+      <c r="B22">
+        <v>1019</v>
+      </c>
+      <c r="C22" t="s">
+        <v>88</v>
+      </c>
+      <c r="D22" t="s">
+        <v>27</v>
+      </c>
+      <c r="E22" t="s">
+        <v>56</v>
+      </c>
+      <c r="F22" t="s">
+        <v>89</v>
+      </c>
+      <c r="G22" t="s">
+        <v>17</v>
+      </c>
+      <c r="H22" t="s">
+        <v>30</v>
+      </c>
+      <c r="I22" t="s">
+        <v>46</v>
+      </c>
+      <c r="J22">
+        <v>66</v>
+      </c>
+      <c r="K22" t="s">
+        <v>73</v>
+      </c>
+      <c r="L22" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12">
+      <c r="A23">
+        <v>20</v>
+      </c>
+      <c r="B23">
+        <v>1020</v>
+      </c>
+      <c r="C23" t="s">
+        <v>91</v>
+      </c>
+      <c r="D23" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" t="s">
+        <v>92</v>
+      </c>
+      <c r="G23" t="s">
+        <v>17</v>
+      </c>
+      <c r="H23" t="s">
+        <v>30</v>
+      </c>
+      <c r="I23" t="s">
+        <v>46</v>
+      </c>
+      <c r="J23">
+        <v>65</v>
+      </c>
+      <c r="K23" t="s">
+        <v>73</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12">
+      <c r="A24">
+        <v>21</v>
+      </c>
+      <c r="B24">
+        <v>1021</v>
+      </c>
+      <c r="C24" t="s">
+        <v>94</v>
+      </c>
+      <c r="D24" t="s">
+        <v>14</v>
+      </c>
+      <c r="E24" t="s">
+        <v>28</v>
+      </c>
+      <c r="F24" t="s">
+        <v>95</v>
+      </c>
+      <c r="G24" t="s">
+        <v>17</v>
+      </c>
+      <c r="H24" t="s">
+        <v>30</v>
+      </c>
+      <c r="I24" t="s">
+        <v>46</v>
+      </c>
+      <c r="J24">
+        <v>64</v>
+      </c>
+      <c r="K24" t="s">
+        <v>96</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12">
+      <c r="A25">
+        <v>22</v>
+      </c>
+      <c r="B25">
+        <v>1022</v>
+      </c>
+      <c r="C25" t="s">
+        <v>98</v>
+      </c>
+      <c r="D25" t="s">
+        <v>27</v>
+      </c>
+      <c r="E25" t="s">
+        <v>34</v>
+      </c>
+      <c r="F25" t="s">
+        <v>99</v>
+      </c>
+      <c r="G25" t="s">
+        <v>17</v>
+      </c>
+      <c r="H25" t="s">
+        <v>30</v>
+      </c>
+      <c r="I25" t="s">
+        <v>46</v>
+      </c>
+      <c r="J25">
+        <v>63</v>
+      </c>
+      <c r="K25" t="s">
+        <v>96</v>
+      </c>
+      <c r="L25" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12">
+      <c r="A26">
+        <v>23</v>
+      </c>
+      <c r="B26">
+        <v>1023</v>
+      </c>
+      <c r="C26" t="s">
+        <v>101</v>
+      </c>
+      <c r="D26" t="s">
+        <v>27</v>
+      </c>
+      <c r="E26" t="s">
+        <v>52</v>
+      </c>
+      <c r="F26" t="s">
+        <v>102</v>
+      </c>
+      <c r="G26" t="s">
+        <v>17</v>
+      </c>
+      <c r="H26" t="s">
+        <v>30</v>
+      </c>
+      <c r="I26" t="s">
+        <v>46</v>
+      </c>
+      <c r="J26">
+        <v>62</v>
+      </c>
+      <c r="K26" t="s">
+        <v>96</v>
+      </c>
+      <c r="L26" s="3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12">
+      <c r="A27">
+        <v>24</v>
+      </c>
+      <c r="B27">
+        <v>1024</v>
+      </c>
+      <c r="C27" t="s">
+        <v>104</v>
+      </c>
+      <c r="D27" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" t="s">
+        <v>56</v>
+      </c>
+      <c r="F27" t="s">
+        <v>105</v>
+      </c>
+      <c r="G27" t="s">
+        <v>17</v>
+      </c>
+      <c r="H27" t="s">
+        <v>30</v>
+      </c>
+      <c r="I27" t="s">
+        <v>46</v>
+      </c>
+      <c r="J27">
+        <v>61</v>
+      </c>
+      <c r="K27" t="s">
+        <v>96</v>
+      </c>
+      <c r="L27" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12">
+      <c r="A28">
+        <v>25</v>
+      </c>
+      <c r="B28">
+        <v>1025</v>
+      </c>
+      <c r="C28" t="s">
+        <v>107</v>
+      </c>
+      <c r="D28" t="s">
+        <v>27</v>
+      </c>
+      <c r="E28" t="s">
+        <v>15</v>
+      </c>
+      <c r="F28" t="s">
+        <v>108</v>
+      </c>
+      <c r="G28" t="s">
+        <v>17</v>
+      </c>
+      <c r="H28" t="s">
+        <v>30</v>
+      </c>
+      <c r="I28" t="s">
+        <v>46</v>
+      </c>
+      <c r="J28">
+        <v>60</v>
+      </c>
+      <c r="K28" t="s">
+        <v>96</v>
+      </c>
+      <c r="L28" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12">
+      <c r="A29">
+        <v>26</v>
+      </c>
+      <c r="B29">
+        <v>1026</v>
+      </c>
+      <c r="C29" t="s">
+        <v>110</v>
+      </c>
+      <c r="D29" t="s">
+        <v>27</v>
+      </c>
+      <c r="E29" t="s">
+        <v>28</v>
+      </c>
+      <c r="F29" t="s">
+        <v>111</v>
+      </c>
+      <c r="G29" t="s">
+        <v>17</v>
+      </c>
+      <c r="H29" t="s">
+        <v>30</v>
+      </c>
+      <c r="I29" t="s">
+        <v>46</v>
+      </c>
+      <c r="J29">
+        <v>59</v>
+      </c>
+      <c r="K29" t="s">
+        <v>96</v>
+      </c>
+      <c r="L29" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
+      <c r="A30">
+        <v>27</v>
+      </c>
+      <c r="B30">
+        <v>1027</v>
+      </c>
+      <c r="C30" t="s">
+        <v>113</v>
+      </c>
+      <c r="D30" t="s">
+        <v>14</v>
+      </c>
+      <c r="E30" t="s">
+        <v>34</v>
+      </c>
+      <c r="F30" t="s">
+        <v>114</v>
+      </c>
+      <c r="G30" t="s">
+        <v>17</v>
+      </c>
+      <c r="H30" t="s">
+        <v>30</v>
+      </c>
+      <c r="I30" t="s">
+        <v>46</v>
+      </c>
+      <c r="J30">
+        <v>58</v>
+      </c>
+      <c r="K30" t="s">
+        <v>96</v>
+      </c>
+      <c r="L30" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
+      <c r="A31">
+        <v>28</v>
+      </c>
+      <c r="B31">
+        <v>1028</v>
+      </c>
+      <c r="C31" t="s">
+        <v>116</v>
+      </c>
+      <c r="D31" t="s">
+        <v>27</v>
+      </c>
+      <c r="E31" t="s">
+        <v>52</v>
+      </c>
+      <c r="F31" t="s">
+        <v>117</v>
+      </c>
+      <c r="G31" t="s">
+        <v>17</v>
+      </c>
+      <c r="H31" t="s">
+        <v>30</v>
+      </c>
+      <c r="I31" t="s">
+        <v>46</v>
+      </c>
+      <c r="J31">
+        <v>57</v>
+      </c>
+      <c r="K31" t="s">
+        <v>118</v>
+      </c>
+      <c r="L31" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12">
+      <c r="A32">
+        <v>29</v>
+      </c>
+      <c r="B32">
+        <v>1029</v>
+      </c>
+      <c r="C32" t="s">
+        <v>120</v>
+      </c>
+      <c r="D32" t="s">
+        <v>27</v>
+      </c>
+      <c r="E32" t="s">
+        <v>56</v>
+      </c>
+      <c r="F32" t="s">
+        <v>121</v>
+      </c>
+      <c r="G32" t="s">
+        <v>17</v>
+      </c>
+      <c r="H32" t="s">
+        <v>30</v>
+      </c>
+      <c r="I32" t="s">
+        <v>46</v>
+      </c>
+      <c r="J32">
+        <v>56</v>
+      </c>
+      <c r="K32" t="s">
+        <v>118</v>
+      </c>
+      <c r="L32" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12">
+      <c r="A33">
+        <v>30</v>
+      </c>
+      <c r="B33">
+        <v>1030</v>
+      </c>
+      <c r="C33" t="s">
+        <v>123</v>
+      </c>
+      <c r="D33" t="s">
+        <v>76</v>
+      </c>
+      <c r="E33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F33" t="s">
+        <v>124</v>
+      </c>
+      <c r="G33" t="s">
+        <v>17</v>
+      </c>
+      <c r="H33" t="s">
+        <v>30</v>
+      </c>
+      <c r="I33" t="s">
+        <v>46</v>
+      </c>
+      <c r="J33">
+        <v>55</v>
+      </c>
+      <c r="K33" t="s">
+        <v>118</v>
+      </c>
+      <c r="L33" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
@@ -816,6 +2012,31 @@
     <hyperlink ref="L6" r:id="rId3"/>
     <hyperlink ref="L7" r:id="rId4"/>
     <hyperlink ref="L8" r:id="rId5"/>
+    <hyperlink ref="L9" r:id="rId6"/>
+    <hyperlink ref="L10" r:id="rId7"/>
+    <hyperlink ref="L11" r:id="rId8"/>
+    <hyperlink ref="L12" r:id="rId9"/>
+    <hyperlink ref="L13" r:id="rId10"/>
+    <hyperlink ref="L14" r:id="rId11"/>
+    <hyperlink ref="L15" r:id="rId12"/>
+    <hyperlink ref="L16" r:id="rId13"/>
+    <hyperlink ref="L17" r:id="rId14"/>
+    <hyperlink ref="L18" r:id="rId15"/>
+    <hyperlink ref="L19" r:id="rId16"/>
+    <hyperlink ref="L20" r:id="rId17"/>
+    <hyperlink ref="L21" r:id="rId18"/>
+    <hyperlink ref="L22" r:id="rId19"/>
+    <hyperlink ref="L23" r:id="rId20"/>
+    <hyperlink ref="L24" r:id="rId21"/>
+    <hyperlink ref="L25" r:id="rId22"/>
+    <hyperlink ref="L26" r:id="rId23"/>
+    <hyperlink ref="L27" r:id="rId24"/>
+    <hyperlink ref="L28" r:id="rId25"/>
+    <hyperlink ref="L29" r:id="rId26"/>
+    <hyperlink ref="L30" r:id="rId27"/>
+    <hyperlink ref="L31" r:id="rId28"/>
+    <hyperlink ref="L32" r:id="rId29"/>
+    <hyperlink ref="L33" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>